<commit_message>
Updated comments at head of file, updated Description and Outcome Message and fixed negative test validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000575/negative/01/data/unit-test-coreid-CG0219-negative.xlsx
+++ b/rules/CORE-000575/negative/01/data/unit-test-coreid-CG0219-negative.xlsx
@@ -596,7 +596,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,6 +628,186 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>$dataset_variables</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>STUDYID, DOMAIN, USUBJID, ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$timing_variables</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>VISITNUM, VISIT, ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>$dataset_variables</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>STUDYID, DOMAIN, USUBJID, ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>$timing_variables</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>VISITNUM, VISIT, ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>$dataset_variables</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>STUDYID, DOMAIN, USUBJID, ...</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>lb.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>$timing_variables</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>VISITNUM, VISIT, ...</t>
         </is>
       </c>
     </row>

</xml_diff>